<commit_message>
feat: drain-meter, club tabs, Hin/Rückrunde sheet + 3 rankings
Frontend:
- budget meter starts full (100) and DRAINS as players are picked (remainingPct)
- per-club tabs (Reiter) above the pool, with picked-count badges; clubFilter

Sheet (make-sheet.mjs):
- Scores split into Hinrunde (MD1-11) + Rückrunde (MD12-22) with
  hinTotal/rueckTotal/playerTotal formula columns
- three standings tabs: Ranking_Gesamt (website default), Ranking_Hin, Ranking_Rueck
- Players + Scores grouped (sorted) by club for easy data entry

Docs:
- SHEET-SETUP.md: new tabs, Hin/Rück usage, mytischtennis Meldung source URLs
  (still empty for 26/27 — wait for finals), updated sanity test
- README + .env.example point at Ranking_Gesamt; tab table refreshed

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plattenplausch-sheet.xlsx
+++ b/plattenplausch-sheet.xlsx
@@ -5,7 +5,9 @@
     <sheet name="Submissions" sheetId="1" r:id="rId1"/>
     <sheet name="Players" sheetId="2" r:id="rId2"/>
     <sheet name="Scores" sheetId="3" r:id="rId3"/>
-    <sheet name="Ranking" sheetId="4" r:id="rId4"/>
+    <sheet name="Ranking_Gesamt" sheetId="4" r:id="rId4"/>
+    <sheet name="Ranking_Hin" sheetId="5" r:id="rId5"/>
+    <sheet name="Ranking_Rueck" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -117,17 +119,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">p001</t>
+          <t xml:space="preserve">p007</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dang Qiu</t>
+          <t xml:space="preserve">Darko Jorgic</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Borussia Düsseldorf</t>
+          <t xml:space="preserve">1. FC Saarbrücken</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -136,23 +138,23 @@
         </is>
       </c>
       <c r="E2">
-        <v>28</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">p002</t>
+          <t xml:space="preserve">p004</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dimitrij Ovtcharov</t>
+          <t xml:space="preserve">Patrick Franziska</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">TTC Neu-Ulm</t>
+          <t xml:space="preserve">1. FC Saarbrücken</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -161,23 +163,23 @@
         </is>
       </c>
       <c r="E3">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">p003</t>
+          <t xml:space="preserve">p017</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Timo Boll</t>
+          <t xml:space="preserve">Wang Yang</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Borussia Düsseldorf</t>
+          <t xml:space="preserve">1. FC Saarbrücken</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -186,98 +188,98 @@
         </is>
       </c>
       <c r="E4">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">p004</t>
+          <t xml:space="preserve">p010</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patrick Franziska</t>
+          <t xml:space="preserve">Benedikt Duda</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. FC Saarbrücken</t>
+          <t xml:space="preserve">ASV Grünwettersbach</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Offensiv</t>
+          <t xml:space="preserve">Allrounder</t>
         </is>
       </c>
       <c r="E5">
-        <v>23</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">p005</t>
+          <t xml:space="preserve">p009</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kay Stumper</t>
+          <t xml:space="preserve">Cedric Meissner</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">TTC Neu-Ulm</t>
+          <t xml:space="preserve">ASV Grünwettersbach</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Allrounder</t>
+          <t xml:space="preserve">Offensiv</t>
         </is>
       </c>
       <c r="E6">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">p006</t>
+          <t xml:space="preserve">p019</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anton Källberg</t>
+          <t xml:space="preserve">Daniel Rinderer</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Borussia Düsseldorf</t>
+          <t xml:space="preserve">ASV Grünwettersbach</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Offensiv</t>
+          <t xml:space="preserve">Abwehr</t>
         </is>
       </c>
       <c r="E7">
-        <v>22</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">p007</t>
+          <t xml:space="preserve">p006</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Darko Jorgic</t>
+          <t xml:space="preserve">Anton Källberg</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. FC Saarbrücken</t>
+          <t xml:space="preserve">Borussia Düsseldorf</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -286,48 +288,48 @@
         </is>
       </c>
       <c r="E8">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">p008</t>
+          <t xml:space="preserve">p001</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ricardo Walther</t>
+          <t xml:space="preserve">Dang Qiu</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">TTC Neu-Ulm</t>
+          <t xml:space="preserve">Borussia Düsseldorf</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Allrounder</t>
+          <t xml:space="preserve">Offensiv</t>
         </is>
       </c>
       <c r="E9">
-        <v>16</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">p009</t>
+          <t xml:space="preserve">p016</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cedric Meissner</t>
+          <t xml:space="preserve">Lim Jonghoon</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">ASV Grünwettersbach</t>
+          <t xml:space="preserve">Borussia Düsseldorf</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -336,23 +338,23 @@
         </is>
       </c>
       <c r="E10">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">p010</t>
+          <t xml:space="preserve">p003</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Benedikt Duda</t>
+          <t xml:space="preserve">Timo Boll</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">ASV Grünwettersbach</t>
+          <t xml:space="preserve">Borussia Düsseldorf</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -361,23 +363,23 @@
         </is>
       </c>
       <c r="E11">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">p011</t>
+          <t xml:space="preserve">p022</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fan Bo Meng</t>
+          <t xml:space="preserve">Filip Zeljko</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">TTF Liebherr Ochsenhausen</t>
+          <t xml:space="preserve">Post SV Mühlhausen</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -386,32 +388,32 @@
         </is>
       </c>
       <c r="E12">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">p012</t>
+          <t xml:space="preserve">p020</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kirill Gerassimenko</t>
+          <t xml:space="preserve">Gerald Pollak</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">TTF Liebherr Ochsenhausen</t>
+          <t xml:space="preserve">Post SV Mühlhausen</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Offensiv</t>
+          <t xml:space="preserve">Allrounder</t>
         </is>
       </c>
       <c r="E13">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14">
@@ -442,12 +444,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">p014</t>
+          <t xml:space="preserve">p021</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ruwen Filus</t>
+          <t xml:space="preserve">Andreas Levenko</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -457,152 +459,152 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abwehr</t>
+          <t xml:space="preserve">Allrounder</t>
         </is>
       </c>
       <c r="E15">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">p015</t>
+          <t xml:space="preserve">p014</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mattias Falck</t>
+          <t xml:space="preserve">Ruwen Filus</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">TTC Neu-Ulm</t>
+          <t xml:space="preserve">TTC Fulda-Maberzell</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Offensiv</t>
+          <t xml:space="preserve">Abwehr</t>
         </is>
       </c>
       <c r="E16">
-        <v>20</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">p016</t>
+          <t xml:space="preserve">p024</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lim Jonghoon</t>
+          <t xml:space="preserve">Vladimir Sidorenko</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Borussia Düsseldorf</t>
+          <t xml:space="preserve">TTC Fulda-Maberzell</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Offensiv</t>
+          <t xml:space="preserve">Allrounder</t>
         </is>
       </c>
       <c r="E17">
-        <v>19</v>
+        <v>11</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">p017</t>
+          <t xml:space="preserve">p002</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wang Yang</t>
+          <t xml:space="preserve">Dimitrij Ovtcharov</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. FC Saarbrücken</t>
+          <t xml:space="preserve">TTC Neu-Ulm</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Allrounder</t>
+          <t xml:space="preserve">Offensiv</t>
         </is>
       </c>
       <c r="E18">
-        <v>18</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">p018</t>
+          <t xml:space="preserve">p005</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tom Closset</t>
+          <t xml:space="preserve">Kay Stumper</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">TTF Liebherr Ochsenhausen</t>
+          <t xml:space="preserve">TTC Neu-Ulm</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Offensiv</t>
+          <t xml:space="preserve">Allrounder</t>
         </is>
       </c>
       <c r="E19">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">p019</t>
+          <t xml:space="preserve">p015</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Daniel Rinderer</t>
+          <t xml:space="preserve">Mattias Falck</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">ASV Grünwettersbach</t>
+          <t xml:space="preserve">TTC Neu-Ulm</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abwehr</t>
+          <t xml:space="preserve">Offensiv</t>
         </is>
       </c>
       <c r="E20">
-        <v>9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">p020</t>
+          <t xml:space="preserve">p008</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gerald Pollak</t>
+          <t xml:space="preserve">Ricardo Walther</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Post SV Mühlhausen</t>
+          <t xml:space="preserve">TTC Neu-Ulm</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -611,48 +613,48 @@
         </is>
       </c>
       <c r="E21">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">p021</t>
+          <t xml:space="preserve">p011</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Andreas Levenko</t>
+          <t xml:space="preserve">Fan Bo Meng</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">TTC Fulda-Maberzell</t>
+          <t xml:space="preserve">TTF Liebherr Ochsenhausen</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Allrounder</t>
+          <t xml:space="preserve">Offensiv</t>
         </is>
       </c>
       <c r="E22">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">p022</t>
+          <t xml:space="preserve">p023</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Filip Zeljko</t>
+          <t xml:space="preserve">Hugo Calderano</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Post SV Mühlhausen</t>
+          <t xml:space="preserve">TTF Liebherr Ochsenhausen</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -661,18 +663,18 @@
         </is>
       </c>
       <c r="E23">
-        <v>9</v>
+        <v>26</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">p023</t>
+          <t xml:space="preserve">p012</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hugo Calderano</t>
+          <t xml:space="preserve">Kirill Gerassimenko</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -686,32 +688,32 @@
         </is>
       </c>
       <c r="E24">
-        <v>26</v>
+        <v>15</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">p024</t>
+          <t xml:space="preserve">p018</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vladimir Sidorenko</t>
+          <t xml:space="preserve">Tom Closset</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">TTC Fulda-Maberzell</t>
+          <t xml:space="preserve">TTF Liebherr Ochsenhausen</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Allrounder</t>
+          <t xml:space="preserve">Offensiv</t>
         </is>
       </c>
       <c r="E25">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -734,115 +736,130 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t xml:space="preserve">club</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t xml:space="preserve">MD1</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t xml:space="preserve">MD2</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t xml:space="preserve">MD3</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t xml:space="preserve">MD4</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t xml:space="preserve">MD5</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t xml:space="preserve">MD6</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t xml:space="preserve">MD7</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t xml:space="preserve">MD8</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t xml:space="preserve">MD9</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t xml:space="preserve">MD10</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t xml:space="preserve">MD11</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t xml:space="preserve">MD12</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t xml:space="preserve">MD13</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t xml:space="preserve">MD14</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t xml:space="preserve">MD15</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t xml:space="preserve">MD16</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t xml:space="preserve">MD17</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t xml:space="preserve">MD18</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t xml:space="preserve">MD19</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t xml:space="preserve">MD20</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t xml:space="preserve">MD21</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t xml:space="preserve">MD22</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hinTotal</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rueckTotal</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
         <is>
           <t xml:space="preserve">playerTotal</t>
         </is>
@@ -851,16 +868,18 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">p001</t>
+          <t xml:space="preserve">p007</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dang Qiu</t>
-        </is>
-      </c>
-      <c r="C2">
-        <v>0</v>
+          <t xml:space="preserve">Darko Jorgic</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. FC Saarbrücken</t>
+        </is>
       </c>
       <c r="D2">
         <v>0</v>
@@ -926,22 +945,33 @@
         <v>0</v>
       </c>
       <c r="Y2">
-        <f>SUM(C2:X2)</f>
+        <v>0</v>
+      </c>
+      <c r="Z2">
+        <f>SUM(D2:N2)</f>
+      </c>
+      <c r="AA2">
+        <f>SUM(O2:Y2)</f>
+      </c>
+      <c r="AB2">
+        <f>Z2+AA2</f>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">p002</t>
+          <t xml:space="preserve">p004</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dimitrij Ovtcharov</t>
-        </is>
-      </c>
-      <c r="C3">
-        <v>0</v>
+          <t xml:space="preserve">Patrick Franziska</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. FC Saarbrücken</t>
+        </is>
       </c>
       <c r="D3">
         <v>0</v>
@@ -1007,22 +1037,33 @@
         <v>0</v>
       </c>
       <c r="Y3">
-        <f>SUM(C3:X3)</f>
+        <v>0</v>
+      </c>
+      <c r="Z3">
+        <f>SUM(D3:N3)</f>
+      </c>
+      <c r="AA3">
+        <f>SUM(O3:Y3)</f>
+      </c>
+      <c r="AB3">
+        <f>Z3+AA3</f>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">p003</t>
+          <t xml:space="preserve">p017</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Timo Boll</t>
-        </is>
-      </c>
-      <c r="C4">
-        <v>0</v>
+          <t xml:space="preserve">Wang Yang</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. FC Saarbrücken</t>
+        </is>
       </c>
       <c r="D4">
         <v>0</v>
@@ -1088,22 +1129,33 @@
         <v>0</v>
       </c>
       <c r="Y4">
-        <f>SUM(C4:X4)</f>
+        <v>0</v>
+      </c>
+      <c r="Z4">
+        <f>SUM(D4:N4)</f>
+      </c>
+      <c r="AA4">
+        <f>SUM(O4:Y4)</f>
+      </c>
+      <c r="AB4">
+        <f>Z4+AA4</f>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">p004</t>
+          <t xml:space="preserve">p010</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patrick Franziska</t>
-        </is>
-      </c>
-      <c r="C5">
-        <v>0</v>
+          <t xml:space="preserve">Benedikt Duda</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ASV Grünwettersbach</t>
+        </is>
       </c>
       <c r="D5">
         <v>0</v>
@@ -1169,22 +1221,33 @@
         <v>0</v>
       </c>
       <c r="Y5">
-        <f>SUM(C5:X5)</f>
+        <v>0</v>
+      </c>
+      <c r="Z5">
+        <f>SUM(D5:N5)</f>
+      </c>
+      <c r="AA5">
+        <f>SUM(O5:Y5)</f>
+      </c>
+      <c r="AB5">
+        <f>Z5+AA5</f>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">p005</t>
+          <t xml:space="preserve">p009</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kay Stumper</t>
-        </is>
-      </c>
-      <c r="C6">
-        <v>0</v>
+          <t xml:space="preserve">Cedric Meissner</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ASV Grünwettersbach</t>
+        </is>
       </c>
       <c r="D6">
         <v>0</v>
@@ -1250,22 +1313,33 @@
         <v>0</v>
       </c>
       <c r="Y6">
-        <f>SUM(C6:X6)</f>
+        <v>0</v>
+      </c>
+      <c r="Z6">
+        <f>SUM(D6:N6)</f>
+      </c>
+      <c r="AA6">
+        <f>SUM(O6:Y6)</f>
+      </c>
+      <c r="AB6">
+        <f>Z6+AA6</f>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">p006</t>
+          <t xml:space="preserve">p019</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anton Källberg</t>
-        </is>
-      </c>
-      <c r="C7">
-        <v>0</v>
+          <t xml:space="preserve">Daniel Rinderer</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ASV Grünwettersbach</t>
+        </is>
       </c>
       <c r="D7">
         <v>0</v>
@@ -1331,22 +1405,33 @@
         <v>0</v>
       </c>
       <c r="Y7">
-        <f>SUM(C7:X7)</f>
+        <v>0</v>
+      </c>
+      <c r="Z7">
+        <f>SUM(D7:N7)</f>
+      </c>
+      <c r="AA7">
+        <f>SUM(O7:Y7)</f>
+      </c>
+      <c r="AB7">
+        <f>Z7+AA7</f>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">p007</t>
+          <t xml:space="preserve">p006</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Darko Jorgic</t>
-        </is>
-      </c>
-      <c r="C8">
-        <v>0</v>
+          <t xml:space="preserve">Anton Källberg</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Borussia Düsseldorf</t>
+        </is>
       </c>
       <c r="D8">
         <v>0</v>
@@ -1412,22 +1497,33 @@
         <v>0</v>
       </c>
       <c r="Y8">
-        <f>SUM(C8:X8)</f>
+        <v>0</v>
+      </c>
+      <c r="Z8">
+        <f>SUM(D8:N8)</f>
+      </c>
+      <c r="AA8">
+        <f>SUM(O8:Y8)</f>
+      </c>
+      <c r="AB8">
+        <f>Z8+AA8</f>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">p008</t>
+          <t xml:space="preserve">p001</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ricardo Walther</t>
-        </is>
-      </c>
-      <c r="C9">
-        <v>0</v>
+          <t xml:space="preserve">Dang Qiu</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Borussia Düsseldorf</t>
+        </is>
       </c>
       <c r="D9">
         <v>0</v>
@@ -1493,22 +1589,33 @@
         <v>0</v>
       </c>
       <c r="Y9">
-        <f>SUM(C9:X9)</f>
+        <v>0</v>
+      </c>
+      <c r="Z9">
+        <f>SUM(D9:N9)</f>
+      </c>
+      <c r="AA9">
+        <f>SUM(O9:Y9)</f>
+      </c>
+      <c r="AB9">
+        <f>Z9+AA9</f>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">p009</t>
+          <t xml:space="preserve">p016</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cedric Meissner</t>
-        </is>
-      </c>
-      <c r="C10">
-        <v>0</v>
+          <t xml:space="preserve">Lim Jonghoon</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Borussia Düsseldorf</t>
+        </is>
       </c>
       <c r="D10">
         <v>0</v>
@@ -1574,22 +1681,33 @@
         <v>0</v>
       </c>
       <c r="Y10">
-        <f>SUM(C10:X10)</f>
+        <v>0</v>
+      </c>
+      <c r="Z10">
+        <f>SUM(D10:N10)</f>
+      </c>
+      <c r="AA10">
+        <f>SUM(O10:Y10)</f>
+      </c>
+      <c r="AB10">
+        <f>Z10+AA10</f>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">p010</t>
+          <t xml:space="preserve">p003</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Benedikt Duda</t>
-        </is>
-      </c>
-      <c r="C11">
-        <v>0</v>
+          <t xml:space="preserve">Timo Boll</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Borussia Düsseldorf</t>
+        </is>
       </c>
       <c r="D11">
         <v>0</v>
@@ -1655,22 +1773,33 @@
         <v>0</v>
       </c>
       <c r="Y11">
-        <f>SUM(C11:X11)</f>
+        <v>0</v>
+      </c>
+      <c r="Z11">
+        <f>SUM(D11:N11)</f>
+      </c>
+      <c r="AA11">
+        <f>SUM(O11:Y11)</f>
+      </c>
+      <c r="AB11">
+        <f>Z11+AA11</f>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">p011</t>
+          <t xml:space="preserve">p022</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fan Bo Meng</t>
-        </is>
-      </c>
-      <c r="C12">
-        <v>0</v>
+          <t xml:space="preserve">Filip Zeljko</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Post SV Mühlhausen</t>
+        </is>
       </c>
       <c r="D12">
         <v>0</v>
@@ -1736,22 +1865,33 @@
         <v>0</v>
       </c>
       <c r="Y12">
-        <f>SUM(C12:X12)</f>
+        <v>0</v>
+      </c>
+      <c r="Z12">
+        <f>SUM(D12:N12)</f>
+      </c>
+      <c r="AA12">
+        <f>SUM(O12:Y12)</f>
+      </c>
+      <c r="AB12">
+        <f>Z12+AA12</f>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">p012</t>
+          <t xml:space="preserve">p020</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kirill Gerassimenko</t>
-        </is>
-      </c>
-      <c r="C13">
-        <v>0</v>
+          <t xml:space="preserve">Gerald Pollak</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Post SV Mühlhausen</t>
+        </is>
       </c>
       <c r="D13">
         <v>0</v>
@@ -1817,7 +1957,16 @@
         <v>0</v>
       </c>
       <c r="Y13">
-        <f>SUM(C13:X13)</f>
+        <v>0</v>
+      </c>
+      <c r="Z13">
+        <f>SUM(D13:N13)</f>
+      </c>
+      <c r="AA13">
+        <f>SUM(O13:Y13)</f>
+      </c>
+      <c r="AB13">
+        <f>Z13+AA13</f>
       </c>
     </row>
     <row r="14">
@@ -1831,8 +1980,10 @@
           <t xml:space="preserve">Steffen Mengel</t>
         </is>
       </c>
-      <c r="C14">
-        <v>0</v>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Post SV Mühlhausen</t>
+        </is>
       </c>
       <c r="D14">
         <v>0</v>
@@ -1898,22 +2049,33 @@
         <v>0</v>
       </c>
       <c r="Y14">
-        <f>SUM(C14:X14)</f>
+        <v>0</v>
+      </c>
+      <c r="Z14">
+        <f>SUM(D14:N14)</f>
+      </c>
+      <c r="AA14">
+        <f>SUM(O14:Y14)</f>
+      </c>
+      <c r="AB14">
+        <f>Z14+AA14</f>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">p014</t>
+          <t xml:space="preserve">p021</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ruwen Filus</t>
-        </is>
-      </c>
-      <c r="C15">
-        <v>0</v>
+          <t xml:space="preserve">Andreas Levenko</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TTC Fulda-Maberzell</t>
+        </is>
       </c>
       <c r="D15">
         <v>0</v>
@@ -1979,22 +2141,33 @@
         <v>0</v>
       </c>
       <c r="Y15">
-        <f>SUM(C15:X15)</f>
+        <v>0</v>
+      </c>
+      <c r="Z15">
+        <f>SUM(D15:N15)</f>
+      </c>
+      <c r="AA15">
+        <f>SUM(O15:Y15)</f>
+      </c>
+      <c r="AB15">
+        <f>Z15+AA15</f>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">p015</t>
+          <t xml:space="preserve">p014</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mattias Falck</t>
-        </is>
-      </c>
-      <c r="C16">
-        <v>0</v>
+          <t xml:space="preserve">Ruwen Filus</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TTC Fulda-Maberzell</t>
+        </is>
       </c>
       <c r="D16">
         <v>0</v>
@@ -2060,22 +2233,33 @@
         <v>0</v>
       </c>
       <c r="Y16">
-        <f>SUM(C16:X16)</f>
+        <v>0</v>
+      </c>
+      <c r="Z16">
+        <f>SUM(D16:N16)</f>
+      </c>
+      <c r="AA16">
+        <f>SUM(O16:Y16)</f>
+      </c>
+      <c r="AB16">
+        <f>Z16+AA16</f>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">p016</t>
+          <t xml:space="preserve">p024</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lim Jonghoon</t>
-        </is>
-      </c>
-      <c r="C17">
-        <v>0</v>
+          <t xml:space="preserve">Vladimir Sidorenko</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TTC Fulda-Maberzell</t>
+        </is>
       </c>
       <c r="D17">
         <v>0</v>
@@ -2141,22 +2325,33 @@
         <v>0</v>
       </c>
       <c r="Y17">
-        <f>SUM(C17:X17)</f>
+        <v>0</v>
+      </c>
+      <c r="Z17">
+        <f>SUM(D17:N17)</f>
+      </c>
+      <c r="AA17">
+        <f>SUM(O17:Y17)</f>
+      </c>
+      <c r="AB17">
+        <f>Z17+AA17</f>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">p017</t>
+          <t xml:space="preserve">p002</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wang Yang</t>
-        </is>
-      </c>
-      <c r="C18">
-        <v>0</v>
+          <t xml:space="preserve">Dimitrij Ovtcharov</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TTC Neu-Ulm</t>
+        </is>
       </c>
       <c r="D18">
         <v>0</v>
@@ -2222,22 +2417,33 @@
         <v>0</v>
       </c>
       <c r="Y18">
-        <f>SUM(C18:X18)</f>
+        <v>0</v>
+      </c>
+      <c r="Z18">
+        <f>SUM(D18:N18)</f>
+      </c>
+      <c r="AA18">
+        <f>SUM(O18:Y18)</f>
+      </c>
+      <c r="AB18">
+        <f>Z18+AA18</f>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">p018</t>
+          <t xml:space="preserve">p005</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tom Closset</t>
-        </is>
-      </c>
-      <c r="C19">
-        <v>0</v>
+          <t xml:space="preserve">Kay Stumper</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TTC Neu-Ulm</t>
+        </is>
       </c>
       <c r="D19">
         <v>0</v>
@@ -2303,22 +2509,33 @@
         <v>0</v>
       </c>
       <c r="Y19">
-        <f>SUM(C19:X19)</f>
+        <v>0</v>
+      </c>
+      <c r="Z19">
+        <f>SUM(D19:N19)</f>
+      </c>
+      <c r="AA19">
+        <f>SUM(O19:Y19)</f>
+      </c>
+      <c r="AB19">
+        <f>Z19+AA19</f>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">p019</t>
+          <t xml:space="preserve">p015</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Daniel Rinderer</t>
-        </is>
-      </c>
-      <c r="C20">
-        <v>0</v>
+          <t xml:space="preserve">Mattias Falck</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TTC Neu-Ulm</t>
+        </is>
       </c>
       <c r="D20">
         <v>0</v>
@@ -2384,22 +2601,33 @@
         <v>0</v>
       </c>
       <c r="Y20">
-        <f>SUM(C20:X20)</f>
+        <v>0</v>
+      </c>
+      <c r="Z20">
+        <f>SUM(D20:N20)</f>
+      </c>
+      <c r="AA20">
+        <f>SUM(O20:Y20)</f>
+      </c>
+      <c r="AB20">
+        <f>Z20+AA20</f>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">p020</t>
+          <t xml:space="preserve">p008</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gerald Pollak</t>
-        </is>
-      </c>
-      <c r="C21">
-        <v>0</v>
+          <t xml:space="preserve">Ricardo Walther</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TTC Neu-Ulm</t>
+        </is>
       </c>
       <c r="D21">
         <v>0</v>
@@ -2465,22 +2693,33 @@
         <v>0</v>
       </c>
       <c r="Y21">
-        <f>SUM(C21:X21)</f>
+        <v>0</v>
+      </c>
+      <c r="Z21">
+        <f>SUM(D21:N21)</f>
+      </c>
+      <c r="AA21">
+        <f>SUM(O21:Y21)</f>
+      </c>
+      <c r="AB21">
+        <f>Z21+AA21</f>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">p021</t>
+          <t xml:space="preserve">p011</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Andreas Levenko</t>
-        </is>
-      </c>
-      <c r="C22">
-        <v>0</v>
+          <t xml:space="preserve">Fan Bo Meng</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TTF Liebherr Ochsenhausen</t>
+        </is>
       </c>
       <c r="D22">
         <v>0</v>
@@ -2546,22 +2785,33 @@
         <v>0</v>
       </c>
       <c r="Y22">
-        <f>SUM(C22:X22)</f>
+        <v>0</v>
+      </c>
+      <c r="Z22">
+        <f>SUM(D22:N22)</f>
+      </c>
+      <c r="AA22">
+        <f>SUM(O22:Y22)</f>
+      </c>
+      <c r="AB22">
+        <f>Z22+AA22</f>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">p022</t>
+          <t xml:space="preserve">p023</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Filip Zeljko</t>
-        </is>
-      </c>
-      <c r="C23">
-        <v>0</v>
+          <t xml:space="preserve">Hugo Calderano</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TTF Liebherr Ochsenhausen</t>
+        </is>
       </c>
       <c r="D23">
         <v>0</v>
@@ -2627,22 +2877,33 @@
         <v>0</v>
       </c>
       <c r="Y23">
-        <f>SUM(C23:X23)</f>
+        <v>0</v>
+      </c>
+      <c r="Z23">
+        <f>SUM(D23:N23)</f>
+      </c>
+      <c r="AA23">
+        <f>SUM(O23:Y23)</f>
+      </c>
+      <c r="AB23">
+        <f>Z23+AA23</f>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">p023</t>
+          <t xml:space="preserve">p012</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hugo Calderano</t>
-        </is>
-      </c>
-      <c r="C24">
-        <v>0</v>
+          <t xml:space="preserve">Kirill Gerassimenko</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TTF Liebherr Ochsenhausen</t>
+        </is>
       </c>
       <c r="D24">
         <v>0</v>
@@ -2708,22 +2969,33 @@
         <v>0</v>
       </c>
       <c r="Y24">
-        <f>SUM(C24:X24)</f>
+        <v>0</v>
+      </c>
+      <c r="Z24">
+        <f>SUM(D24:N24)</f>
+      </c>
+      <c r="AA24">
+        <f>SUM(O24:Y24)</f>
+      </c>
+      <c r="AB24">
+        <f>Z24+AA24</f>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">p024</t>
+          <t xml:space="preserve">p018</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vladimir Sidorenko</t>
-        </is>
-      </c>
-      <c r="C25">
-        <v>0</v>
+          <t xml:space="preserve">Tom Closset</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TTF Liebherr Ochsenhausen</t>
+        </is>
       </c>
       <c r="D25">
         <v>0</v>
@@ -2789,7 +3061,16 @@
         <v>0</v>
       </c>
       <c r="Y25">
-        <f>SUM(C25:X25)</f>
+        <v>0</v>
+      </c>
+      <c r="Z25">
+        <f>SUM(D25:N25)</f>
+      </c>
+      <c r="AA25">
+        <f>SUM(O25:Y25)</f>
+      </c>
+      <c r="AB25">
+        <f>Z25+AA25</f>
       </c>
     </row>
   </sheetData>
@@ -2860,7 +3141,161 @@
         <f>MAP(Submissions!$C$2:$C,Submissions!$K$2:$K,Submissions!$M$2:$M,LAMBDA(tn,cf,ss,IF(tn="","",IF(AND(cf=TRUE,ss&lt;&gt;TRUE),TRUE,FALSE))))</f>
       </c>
       <c r="F2">
-        <f>BYROW(Submissions!$D$2:$I,LAMBDA(row,IF(INDEX(row,1,1)="","",SUMPRODUCT(IFERROR(XLOOKUP(row,Scores!$A$2:$A$25,Scores!$Y$2:$Y$25),0)))))</f>
+        <f>BYROW(Submissions!$D$2:$I,LAMBDA(row,IF(INDEX(row,1,1)="","",SUMPRODUCT(IFERROR(XLOOKUP(row,Scores!$A$2:$A$25,Scores!$AB$2:$AB$25),0)))))</f>
+      </c>
+      <c r="G2">
+        <f>ARRAYFORMULA(IF(Submissions!$C$2:$C="","",Submissions!$A$2:$A))</f>
+      </c>
+      <c r="H2">
+        <f>ARRAYFORMULA(IF(Submissions!$C$2:$C="","",Submissions!$C$2:$C))</f>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">teamName</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">total</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">active</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">teamTotal</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">submittedAt</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">teamNameSrc</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <f>IF(COUNTA(B2:B)=0,"",SEQUENCE(COUNTA(B2:B)))</f>
+      </c>
+      <c r="B2">
+        <f>IFERROR(INDEX(SORT(FILTER({$H$2:$H,$F$2:$F,$G$2:$G},$E$2:$E=TRUE),2,FALSE,3,TRUE,1,TRUE),0,1),"")</f>
+      </c>
+      <c r="C2">
+        <f>IFERROR(INDEX(SORT(FILTER({$H$2:$H,$F$2:$F,$G$2:$G},$E$2:$E=TRUE),2,FALSE,3,TRUE,1,TRUE),0,2),"")</f>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E2">
+        <f>MAP(Submissions!$C$2:$C,Submissions!$K$2:$K,Submissions!$M$2:$M,LAMBDA(tn,cf,ss,IF(tn="","",IF(AND(cf=TRUE,ss&lt;&gt;TRUE),TRUE,FALSE))))</f>
+      </c>
+      <c r="F2">
+        <f>BYROW(Submissions!$D$2:$I,LAMBDA(row,IF(INDEX(row,1,1)="","",SUMPRODUCT(IFERROR(XLOOKUP(row,Scores!$A$2:$A$25,Scores!$Z$2:$Z$25),0)))))</f>
+      </c>
+      <c r="G2">
+        <f>ARRAYFORMULA(IF(Submissions!$C$2:$C="","",Submissions!$A$2:$A))</f>
+      </c>
+      <c r="H2">
+        <f>ARRAYFORMULA(IF(Submissions!$C$2:$C="","",Submissions!$C$2:$C))</f>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">teamName</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">total</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">active</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">teamTotal</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">submittedAt</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">teamNameSrc</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <f>IF(COUNTA(B2:B)=0,"",SEQUENCE(COUNTA(B2:B)))</f>
+      </c>
+      <c r="B2">
+        <f>IFERROR(INDEX(SORT(FILTER({$H$2:$H,$F$2:$F,$G$2:$G},$E$2:$E=TRUE),2,FALSE,3,TRUE,1,TRUE),0,1),"")</f>
+      </c>
+      <c r="C2">
+        <f>IFERROR(INDEX(SORT(FILTER({$H$2:$H,$F$2:$F,$G$2:$G},$E$2:$E=TRUE),2,FALSE,3,TRUE,1,TRUE),0,2),"")</f>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E2">
+        <f>MAP(Submissions!$C$2:$C,Submissions!$K$2:$K,Submissions!$M$2:$M,LAMBDA(tn,cf,ss,IF(tn="","",IF(AND(cf=TRUE,ss&lt;&gt;TRUE),TRUE,FALSE))))</f>
+      </c>
+      <c r="F2">
+        <f>BYROW(Submissions!$D$2:$I,LAMBDA(row,IF(INDEX(row,1,1)="","",SUMPRODUCT(IFERROR(XLOOKUP(row,Scores!$A$2:$A$25,Scores!$AA$2:$AA$25),0)))))</f>
       </c>
       <c r="G2">
         <f>ARRAYFORMULA(IF(Submissions!$C$2:$C="","",Submissions!$A$2:$A))</f>

</xml_diff>

<commit_message>
fix(sheet): bound ranking ranges so MAP/BYROW evaluate in Sheets
Open-ended column ranges ($2:$C) made MAP/BYROW receive unequal-length
inputs and the Gesamt rowTotal used MAP+SEQUENCE+INDEX-by-i — both throw in
Google Sheets, cascading errors to every ranking cell.

- bound all Submissions + helper ranges to a fixed MAXSUB=1000 (rows 2..1001)
- Gesamt rowTotal: replace MAP+SEQUENCE+INDEX with ARRAYFORMULA(IF(round,...))
  over two bounded BYROW pick-sums (hin/rück)
- regenerated plattenplausch-sheet.xlsx
- verified logic in a simulation: test scenario yields Hin=10 Rueck=7 Gesamt=17

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plattenplausch-sheet.xlsx
+++ b/plattenplausch-sheet.xlsx
@@ -6250,10 +6250,10 @@
         <f>IF(COUNTA(B2:B)=0,"",SEQUENCE(COUNTA(B2:B)))</f>
       </c>
       <c r="B2">
-        <f>IFERROR(INDEX(SORT(FILTER({$M$2:$M,$L$2:$L,$N$2:$N},$K$2:$K&lt;&gt;""),2,FALSE,3,TRUE,1,TRUE),0,1),"")</f>
+        <f>IFERROR(INDEX(SORT(FILTER({$M$2:$M$1001,$L$2:$L$1001,$N$2:$N$1001},$K$2:$K$1001&lt;&gt;""),2,FALSE,3,TRUE,1,TRUE),0,1),"")</f>
       </c>
       <c r="C2">
-        <f>IFERROR(INDEX(SORT(FILTER({$M$2:$M,$L$2:$L,$N$2:$N},$K$2:$K&lt;&gt;""),2,FALSE,3,TRUE,1,TRUE),0,2),"")</f>
+        <f>IFERROR(INDEX(SORT(FILTER({$M$2:$M$1001,$L$2:$L$1001,$N$2:$N$1001},$K$2:$K$1001&lt;&gt;""),2,FALSE,3,TRUE,1,TRUE),0,2),"")</f>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -6261,19 +6261,19 @@
         </is>
       </c>
       <c r="E2">
-        <f>MAP(Submissions!$C$2:$C,Submissions!$L$2:$L,Submissions!$N$2:$N,LAMBDA(tn,cf,ss,IF(tn="","",IF(AND(cf=TRUE,ss&lt;&gt;TRUE),TRUE,FALSE))))</f>
+        <f>MAP(Submissions!$C$2:$C$1001,Submissions!$L$2:$L$1001,Submissions!$N$2:$N$1001,LAMBDA(tn,cf,ss,IF(tn="",FALSE,IF(AND(cf=TRUE,ss&lt;&gt;TRUE),TRUE,FALSE))))</f>
       </c>
       <c r="F2">
-        <f>ARRAYFORMULA(IF($E$2:$E=TRUE,Submissions!$B$2:$B,""))</f>
+        <f>ARRAYFORMULA(IF($E$2:$E$1001=TRUE,Submissions!$B$2:$B$1001,""))</f>
       </c>
       <c r="G2">
-        <f>MAP(Submissions!$D$2:$D,SEQUENCE(ROWS(Submissions!$D$2:$D)),LAMBDA(rd,i,IF(INDEX($E$2:$E,i)&lt;&gt;TRUE,"",LET(picks,INDEX(Submissions!$E$2:$J,i,0),IF(rd="HIN",SUMPRODUCT(IFERROR(XLOOKUP(picks,Scores!$A$2:$A$49,Scores!$AA$2:$AA$49),0)),IF(rd="RUECK",SUMPRODUCT(IFERROR(XLOOKUP(picks,Scores!$A$2:$A$49,Scores!$AB$2:$AB$49),0)),0))))))</f>
+        <f>ARRAYFORMULA(IF($E$2:$E$1001&lt;&gt;TRUE,"",IF(Submissions!$D$2:$D$1001="HIN",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores!$A$2:$A$49,Scores!$AA$2:$AA$49),0))))),IF(Submissions!$D$2:$D$1001="RUECK",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores!$A$2:$A$49,Scores!$AB$2:$AB$49),0))))),0))))</f>
       </c>
       <c r="H2">
-        <f>ARRAYFORMULA(IF($E$2:$E=TRUE,Submissions!$C$2:$C,""))</f>
+        <f>ARRAYFORMULA(IF($E$2:$E$1001=TRUE,Submissions!$C$2:$C$1001,""))</f>
       </c>
       <c r="I2">
-        <f>ARRAYFORMULA(IF($E$2:$E=TRUE,Submissions!$A$2:$A,""))</f>
+        <f>ARRAYFORMULA(IF($E$2:$E$1001=TRUE,Submissions!$A$2:$A$1001,""))</f>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -6281,16 +6281,16 @@
         </is>
       </c>
       <c r="K2">
-        <f>IFERROR(UNIQUE(FILTER($F$2:$F,$F$2:$F&lt;&gt;"")),"")</f>
+        <f>IFERROR(UNIQUE(FILTER($F$2:$F$1001,$F$2:$F$1001&lt;&gt;"")),"")</f>
       </c>
       <c r="L2">
-        <f>MAP($K$2:$K,LAMBDA(e,IF(e="","",SUMIF($F$2:$F,e,$G$2:$G))))</f>
+        <f>MAP($K$2:$K$1001,LAMBDA(e,IF(e="","",SUMIF($F$2:$F$1001,e,$G$2:$G$1001))))</f>
       </c>
       <c r="M2">
-        <f>MAP($K$2:$K,LAMBDA(e,IF(e="","",IFERROR(INDEX(FILTER($H$2:$H,$F$2:$F=e),1),""))))</f>
+        <f>MAP($K$2:$K$1001,LAMBDA(e,IF(e="","",IFERROR(INDEX(FILTER($H$2:$H$1001,$F$2:$F$1001=e),1),""))))</f>
       </c>
       <c r="N2">
-        <f>MAP($K$2:$K,LAMBDA(e,IF(e="","",MINIFS($I$2:$I,$F$2:$F,e))))</f>
+        <f>MAP($K$2:$K$1001,LAMBDA(e,IF(e="","",MINIFS($I$2:$I$1001,$F$2:$F$1001,e))))</f>
       </c>
     </row>
   </sheetData>
@@ -6347,10 +6347,10 @@
         <f>IF(COUNTA(B2:B)=0,"",SEQUENCE(COUNTA(B2:B)))</f>
       </c>
       <c r="B2">
-        <f>IFERROR(INDEX(SORT(FILTER({$H$2:$H,$F$2:$F,$G$2:$G},$E$2:$E=TRUE),2,FALSE,3,TRUE,1,TRUE),0,1),"")</f>
+        <f>IFERROR(INDEX(SORT(FILTER({$H$2:$H$1001,$F$2:$F$1001,$G$2:$G$1001},$E$2:$E$1001=TRUE),2,FALSE,3,TRUE,1,TRUE),0,1),"")</f>
       </c>
       <c r="C2">
-        <f>IFERROR(INDEX(SORT(FILTER({$H$2:$H,$F$2:$F,$G$2:$G},$E$2:$E=TRUE),2,FALSE,3,TRUE,1,TRUE),0,2),"")</f>
+        <f>IFERROR(INDEX(SORT(FILTER({$H$2:$H$1001,$F$2:$F$1001,$G$2:$G$1001},$E$2:$E$1001=TRUE),2,FALSE,3,TRUE,1,TRUE),0,2),"")</f>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -6358,16 +6358,16 @@
         </is>
       </c>
       <c r="E2">
-        <f>MAP(Submissions!$C$2:$C,Submissions!$L$2:$L,Submissions!$N$2:$N,Submissions!$D$2:$D,LAMBDA(tn,cf,ss,rd,IF(tn="","",IF(AND(cf=TRUE,ss&lt;&gt;TRUE,rd="HIN"),TRUE,FALSE))))</f>
+        <f>MAP(Submissions!$C$2:$C$1001,Submissions!$L$2:$L$1001,Submissions!$N$2:$N$1001,Submissions!$D$2:$D$1001,LAMBDA(tn,cf,ss,rd,IF(tn="",FALSE,IF(AND(cf=TRUE,ss&lt;&gt;TRUE,rd="HIN"),TRUE,FALSE))))</f>
       </c>
       <c r="F2">
-        <f>BYROW(Submissions!$E$2:$J,LAMBDA(row,IF(INDEX(row,1,1)="","",SUMPRODUCT(IFERROR(XLOOKUP(row,Scores!$A$2:$A$49,Scores!$AA$2:$AA$49),0)))))</f>
+        <f>BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores!$A$2:$A$49,Scores!$AA$2:$AA$49),0)))))</f>
       </c>
       <c r="G2">
-        <f>ARRAYFORMULA(IF(Submissions!$C$2:$C="","",Submissions!$A$2:$A))</f>
+        <f>ARRAYFORMULA(IF(Submissions!$C$2:$C$1001="","",Submissions!$A$2:$A$1001))</f>
       </c>
       <c r="H2">
-        <f>ARRAYFORMULA(IF(Submissions!$C$2:$C="","",Submissions!$C$2:$C))</f>
+        <f>ARRAYFORMULA(IF(Submissions!$C$2:$C$1001="","",Submissions!$C$2:$C$1001))</f>
       </c>
     </row>
   </sheetData>
@@ -6424,10 +6424,10 @@
         <f>IF(COUNTA(B2:B)=0,"",SEQUENCE(COUNTA(B2:B)))</f>
       </c>
       <c r="B2">
-        <f>IFERROR(INDEX(SORT(FILTER({$H$2:$H,$F$2:$F,$G$2:$G},$E$2:$E=TRUE),2,FALSE,3,TRUE,1,TRUE),0,1),"")</f>
+        <f>IFERROR(INDEX(SORT(FILTER({$H$2:$H$1001,$F$2:$F$1001,$G$2:$G$1001},$E$2:$E$1001=TRUE),2,FALSE,3,TRUE,1,TRUE),0,1),"")</f>
       </c>
       <c r="C2">
-        <f>IFERROR(INDEX(SORT(FILTER({$H$2:$H,$F$2:$F,$G$2:$G},$E$2:$E=TRUE),2,FALSE,3,TRUE,1,TRUE),0,2),"")</f>
+        <f>IFERROR(INDEX(SORT(FILTER({$H$2:$H$1001,$F$2:$F$1001,$G$2:$G$1001},$E$2:$E$1001=TRUE),2,FALSE,3,TRUE,1,TRUE),0,2),"")</f>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -6435,16 +6435,16 @@
         </is>
       </c>
       <c r="E2">
-        <f>MAP(Submissions!$C$2:$C,Submissions!$L$2:$L,Submissions!$N$2:$N,Submissions!$D$2:$D,LAMBDA(tn,cf,ss,rd,IF(tn="","",IF(AND(cf=TRUE,ss&lt;&gt;TRUE,rd="RUECK"),TRUE,FALSE))))</f>
+        <f>MAP(Submissions!$C$2:$C$1001,Submissions!$L$2:$L$1001,Submissions!$N$2:$N$1001,Submissions!$D$2:$D$1001,LAMBDA(tn,cf,ss,rd,IF(tn="",FALSE,IF(AND(cf=TRUE,ss&lt;&gt;TRUE,rd="RUECK"),TRUE,FALSE))))</f>
       </c>
       <c r="F2">
-        <f>BYROW(Submissions!$E$2:$J,LAMBDA(row,IF(INDEX(row,1,1)="","",SUMPRODUCT(IFERROR(XLOOKUP(row,Scores!$A$2:$A$49,Scores!$AB$2:$AB$49),0)))))</f>
+        <f>BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores!$A$2:$A$49,Scores!$AB$2:$AB$49),0)))))</f>
       </c>
       <c r="G2">
-        <f>ARRAYFORMULA(IF(Submissions!$C$2:$C="","",Submissions!$A$2:$A))</f>
+        <f>ARRAYFORMULA(IF(Submissions!$C$2:$C$1001="","",Submissions!$A$2:$A$1001))</f>
       </c>
       <c r="H2">
-        <f>ARRAYFORMULA(IF(Submissions!$C$2:$C="","",Submissions!$C$2:$C))</f>
+        <f>ARRAYFORMULA(IF(Submissions!$C$2:$C$1001="","",Submissions!$C$2:$C$1001))</f>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(sheet): rank spills in lockstep with teamName (no blank tie rows)
SEQUENCE(COUNTA(B2:B)) left the 2nd tied team's rank cell blank. Replace with a
SCAN running-count over the bounded B column: filled rows get sequential
1,2,3… (ties broken upstream by submittedAt then name), blank rows stay empty.
Applied to all three Ranking tabs.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plattenplausch-sheet.xlsx
+++ b/plattenplausch-sheet.xlsx
@@ -4150,7 +4150,7 @@
     </row>
     <row r="2">
       <c r="A2">
-        <f>IF(COUNTA(B2:B)=0,"",SEQUENCE(COUNTA(B2:B)))</f>
+        <f>ARRAYFORMULA(IF($B$2:$B$1001="","",SCAN(0,$B$2:$B$1001,LAMBDA(acc,v,IF(v="",acc,acc+1)))))</f>
       </c>
       <c r="B2">
         <f>IFERROR(INDEX(SORT(FILTER({$M$2:$M$1001,$L$2:$L$1001,$N$2:$N$1001},$K$2:$K$1001&lt;&gt;""),2,FALSE,3,TRUE,1,TRUE),0,1),"")</f>
@@ -4247,7 +4247,7 @@
     </row>
     <row r="2">
       <c r="A2">
-        <f>IF(COUNTA(B2:B)=0,"",SEQUENCE(COUNTA(B2:B)))</f>
+        <f>ARRAYFORMULA(IF($B$2:$B$1001="","",SCAN(0,$B$2:$B$1001,LAMBDA(acc,v,IF(v="",acc,acc+1)))))</f>
       </c>
       <c r="B2">
         <f>IFERROR(INDEX(SORT(FILTER({$H$2:$H$1001,$F$2:$F$1001,$G$2:$G$1001},$E$2:$E$1001=TRUE),2,FALSE,3,TRUE,1,TRUE),0,1),"")</f>
@@ -4324,7 +4324,7 @@
     </row>
     <row r="2">
       <c r="A2">
-        <f>IF(COUNTA(B2:B)=0,"",SEQUENCE(COUNTA(B2:B)))</f>
+        <f>ARRAYFORMULA(IF($B$2:$B$1001="","",SCAN(0,$B$2:$B$1001,LAMBDA(acc,v,IF(v="",acc,acc+1)))))</f>
       </c>
       <c r="B2">
         <f>IFERROR(INDEX(SORT(FILTER({$H$2:$H$1001,$F$2:$F$1001,$G$2:$G$1001},$E$2:$E$1001=TRUE),2,FALSE,3,TRUE,1,TRUE),0,1),"")</f>

</xml_diff>

<commit_message>
fix(sheet,privacy): keep email off Ranking_Gesamt entirely
Ranking_Gesamt previously held email in helper columns (F/K), so the published
gviz endpoint could leak addresses. Rewrite the whole email-join inside a single
LET in B2/C2 — email is a LET-local intermediate, never written to a cell. Tab
now has ONLY rank|teamName|total (3 cols, no helpers). Per-round tabs already
carry no email. Verified: no Ranking tab outputs an address; logic still yields
Test=17 / Test2=10.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plattenplausch-sheet.xlsx
+++ b/plattenplausch-sheet.xlsx
@@ -4092,108 +4092,16 @@
           <t xml:space="preserve">total</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">active</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">email</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rowTotal</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">teamNameSrc</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">submittedAt</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">uEmail</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">uTotal</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">uName</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">uEarliest</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2">
         <f>ARRAYFORMULA(IF($B$2:$B$1001="","",SCAN(0,$B$2:$B$1001,LAMBDA(acc,v,IF(v="",acc,acc+1)))))</f>
       </c>
       <c r="B2">
-        <f>IFERROR(INDEX(SORT(FILTER({$M$2:$M$1001,$L$2:$L$1001,$N$2:$N$1001},$K$2:$K$1001&lt;&gt;""),2,FALSE,3,TRUE,1,TRUE),0,1),"")</f>
+        <f>IFERROR(LET(act,MAP(Submissions!$C$2:$C$1001,Submissions!$L$2:$L$1001,Submissions!$N$2:$N$1001,LAMBDA(tn,cf,ss,IF(tn="",FALSE,AND(cf=TRUE,ss&lt;&gt;TRUE)))),eml,IF(act,Submissions!$B$2:$B$1001,""),tot,IF(act,IF(Submissions!$D$2:$D$1001="HIN",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores_Hin!$A$2:$A$25,Scores_Hin!$O$2:$O$25),0))))),IF(Submissions!$D$2:$D$1001="RUECK",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores_Rueck!$A$2:$A$25,Scores_Rueck!$O$2:$O$25),0))))),0)),""),nm,IF(act,Submissions!$C$2:$C$1001,""),sub,IF(act,Submissions!$A$2:$A$1001,""),ue,UNIQUE(FILTER(eml,eml&lt;&gt;"")),uTot,MAP(ue,LAMBDA(e,SUMIF(eml,e,tot))),uName,MAP(ue,LAMBDA(e,INDEX(FILTER(nm,eml=e),1))),uEarl,MAP(ue,LAMBDA(e,MINIFS(sub,eml,e))),sorted,SORT(HSTACK(uName,uTot,uEarl),2,FALSE,3,TRUE,1,TRUE),INDEX(sorted,0,1)),"")</f>
       </c>
       <c r="C2">
-        <f>IFERROR(INDEX(SORT(FILTER({$M$2:$M$1001,$L$2:$L$1001,$N$2:$N$1001},$K$2:$K$1001&lt;&gt;""),2,FALSE,3,TRUE,1,TRUE),0,2),"")</f>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E2">
-        <f>MAP(Submissions!$C$2:$C$1001,Submissions!$L$2:$L$1001,Submissions!$N$2:$N$1001,LAMBDA(tn,cf,ss,IF(tn="",FALSE,IF(AND(cf=TRUE,ss&lt;&gt;TRUE),TRUE,FALSE))))</f>
-      </c>
-      <c r="F2">
-        <f>ARRAYFORMULA(IF($E$2:$E$1001=TRUE,Submissions!$B$2:$B$1001,""))</f>
-      </c>
-      <c r="G2">
-        <f>ARRAYFORMULA(IF($E$2:$E$1001&lt;&gt;TRUE,"",IF(Submissions!$D$2:$D$1001="HIN",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores_Hin!$A$2:$A$25,Scores_Hin!$O$2:$O$25),0))))),IF(Submissions!$D$2:$D$1001="RUECK",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores_Rueck!$A$2:$A$25,Scores_Rueck!$O$2:$O$25),0))))),0))))</f>
-      </c>
-      <c r="H2">
-        <f>ARRAYFORMULA(IF($E$2:$E$1001=TRUE,Submissions!$C$2:$C$1001,""))</f>
-      </c>
-      <c r="I2">
-        <f>ARRAYFORMULA(IF($E$2:$E$1001=TRUE,Submissions!$A$2:$A$1001,""))</f>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K2">
-        <f>IFERROR(UNIQUE(FILTER($F$2:$F$1001,$F$2:$F$1001&lt;&gt;"")),"")</f>
-      </c>
-      <c r="L2">
-        <f>MAP($K$2:$K$1001,LAMBDA(e,IF(e="","",SUMIF($F$2:$F$1001,e,$G$2:$G$1001))))</f>
-      </c>
-      <c r="M2">
-        <f>MAP($K$2:$K$1001,LAMBDA(e,IF(e="","",IFERROR(INDEX(FILTER($H$2:$H$1001,$F$2:$F$1001=e),1),""))))</f>
-      </c>
-      <c r="N2">
-        <f>MAP($K$2:$K$1001,LAMBDA(e,IF(e="","",MINIFS($I$2:$I$1001,$F$2:$F$1001,e))))</f>
+        <f>IFERROR(LET(act,MAP(Submissions!$C$2:$C$1001,Submissions!$L$2:$L$1001,Submissions!$N$2:$N$1001,LAMBDA(tn,cf,ss,IF(tn="",FALSE,AND(cf=TRUE,ss&lt;&gt;TRUE)))),eml,IF(act,Submissions!$B$2:$B$1001,""),tot,IF(act,IF(Submissions!$D$2:$D$1001="HIN",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores_Hin!$A$2:$A$25,Scores_Hin!$O$2:$O$25),0))))),IF(Submissions!$D$2:$D$1001="RUECK",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores_Rueck!$A$2:$A$25,Scores_Rueck!$O$2:$O$25),0))))),0)),""),nm,IF(act,Submissions!$C$2:$C$1001,""),sub,IF(act,Submissions!$A$2:$A$1001,""),ue,UNIQUE(FILTER(eml,eml&lt;&gt;"")),uTot,MAP(ue,LAMBDA(e,SUMIF(eml,e,tot))),uName,MAP(ue,LAMBDA(e,INDEX(FILTER(nm,eml=e),1))),uEarl,MAP(ue,LAMBDA(e,MINIFS(sub,eml,e))),sorted,SORT(HSTACK(uName,uTot,uEarl),2,FALSE,3,TRUE,1,TRUE),INDEX(sorted,0,2)),"")</f>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(sheet): Ranking_Gesamt total was blank (SUMIF on array → SUMPRODUCT)
The privacy-LET rewrite summed per-email totals with SUMIF(eml,e,tot), but
SUMIF's sum_range is unreliable on an in-memory (LET-local) array — name column
resolved, total column came back blank. Use array-native SUMPRODUCT((eml=e)*tot)
and make  default to 0 (not "") for inactive rows so it stays numeric.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plattenplausch-sheet.xlsx
+++ b/plattenplausch-sheet.xlsx
@@ -4098,10 +4098,10 @@
         <f>ARRAYFORMULA(IF($B$2:$B$1001="","",SCAN(0,$B$2:$B$1001,LAMBDA(acc,v,IF(v="",acc,acc+1)))))</f>
       </c>
       <c r="B2">
-        <f>IFERROR(LET(act,MAP(Submissions!$C$2:$C$1001,Submissions!$L$2:$L$1001,Submissions!$N$2:$N$1001,LAMBDA(tn,cf,ss,IF(tn="",FALSE,AND(cf=TRUE,ss&lt;&gt;TRUE)))),eml,IF(act,Submissions!$B$2:$B$1001,""),tot,IF(act,IF(Submissions!$D$2:$D$1001="HIN",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores_Hin!$A$2:$A$25,Scores_Hin!$O$2:$O$25),0))))),IF(Submissions!$D$2:$D$1001="RUECK",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores_Rueck!$A$2:$A$25,Scores_Rueck!$O$2:$O$25),0))))),0)),""),nm,IF(act,Submissions!$C$2:$C$1001,""),sub,IF(act,Submissions!$A$2:$A$1001,""),ue,UNIQUE(FILTER(eml,eml&lt;&gt;"")),uTot,MAP(ue,LAMBDA(e,SUMIF(eml,e,tot))),uName,MAP(ue,LAMBDA(e,INDEX(FILTER(nm,eml=e),1))),uEarl,MAP(ue,LAMBDA(e,MINIFS(sub,eml,e))),sorted,SORT(HSTACK(uName,uTot,uEarl),2,FALSE,3,TRUE,1,TRUE),INDEX(sorted,0,1)),"")</f>
+        <f>IFERROR(LET(act,MAP(Submissions!$C$2:$C$1001,Submissions!$L$2:$L$1001,Submissions!$N$2:$N$1001,LAMBDA(tn,cf,ss,IF(tn="",FALSE,AND(cf=TRUE,ss&lt;&gt;TRUE)))),eml,IF(act,Submissions!$B$2:$B$1001,""),tot,IF(act,IF(Submissions!$D$2:$D$1001="HIN",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores_Hin!$A$2:$A$25,Scores_Hin!$O$2:$O$25),0))))),IF(Submissions!$D$2:$D$1001="RUECK",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores_Rueck!$A$2:$A$25,Scores_Rueck!$O$2:$O$25),0))))),0)),0),nm,IF(act,Submissions!$C$2:$C$1001,""),sub,IF(act,Submissions!$A$2:$A$1001,""),ue,UNIQUE(FILTER(eml,eml&lt;&gt;"")),uTot,MAP(ue,LAMBDA(e,SUMPRODUCT((eml=e)*IF(ISNUMBER(tot),tot,0)))),uName,MAP(ue,LAMBDA(e,INDEX(FILTER(nm,eml=e),1))),uEarl,MAP(ue,LAMBDA(e,MINIFS(sub,eml,e))),sorted,SORT(HSTACK(uName,uTot,uEarl),2,FALSE,3,TRUE,1,TRUE),INDEX(sorted,0,1)),"")</f>
       </c>
       <c r="C2">
-        <f>IFERROR(LET(act,MAP(Submissions!$C$2:$C$1001,Submissions!$L$2:$L$1001,Submissions!$N$2:$N$1001,LAMBDA(tn,cf,ss,IF(tn="",FALSE,AND(cf=TRUE,ss&lt;&gt;TRUE)))),eml,IF(act,Submissions!$B$2:$B$1001,""),tot,IF(act,IF(Submissions!$D$2:$D$1001="HIN",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores_Hin!$A$2:$A$25,Scores_Hin!$O$2:$O$25),0))))),IF(Submissions!$D$2:$D$1001="RUECK",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores_Rueck!$A$2:$A$25,Scores_Rueck!$O$2:$O$25),0))))),0)),""),nm,IF(act,Submissions!$C$2:$C$1001,""),sub,IF(act,Submissions!$A$2:$A$1001,""),ue,UNIQUE(FILTER(eml,eml&lt;&gt;"")),uTot,MAP(ue,LAMBDA(e,SUMIF(eml,e,tot))),uName,MAP(ue,LAMBDA(e,INDEX(FILTER(nm,eml=e),1))),uEarl,MAP(ue,LAMBDA(e,MINIFS(sub,eml,e))),sorted,SORT(HSTACK(uName,uTot,uEarl),2,FALSE,3,TRUE,1,TRUE),INDEX(sorted,0,2)),"")</f>
+        <f>IFERROR(LET(act,MAP(Submissions!$C$2:$C$1001,Submissions!$L$2:$L$1001,Submissions!$N$2:$N$1001,LAMBDA(tn,cf,ss,IF(tn="",FALSE,AND(cf=TRUE,ss&lt;&gt;TRUE)))),eml,IF(act,Submissions!$B$2:$B$1001,""),tot,IF(act,IF(Submissions!$D$2:$D$1001="HIN",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores_Hin!$A$2:$A$25,Scores_Hin!$O$2:$O$25),0))))),IF(Submissions!$D$2:$D$1001="RUECK",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores_Rueck!$A$2:$A$25,Scores_Rueck!$O$2:$O$25),0))))),0)),0),nm,IF(act,Submissions!$C$2:$C$1001,""),sub,IF(act,Submissions!$A$2:$A$1001,""),ue,UNIQUE(FILTER(eml,eml&lt;&gt;"")),uTot,MAP(ue,LAMBDA(e,SUMPRODUCT((eml=e)*IF(ISNUMBER(tot),tot,0)))),uName,MAP(ue,LAMBDA(e,INDEX(FILTER(nm,eml=e),1))),uEarl,MAP(ue,LAMBDA(e,MINIFS(sub,eml,e))),sorted,SORT(HSTACK(uName,uTot,uEarl),2,FALSE,3,TRUE,1,TRUE),INDEX(sorted,0,2)),"")</f>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(sheet): Ranking_Gesamt leaked unconfirmed teams (strict act=TRUE)
Ranking_Hin/Rueck filtered correctly (FILTER on a cell column =TRUE), but
Ranking_Gesamt computed the active mask inside a LET and consumed it via
IF(act,...) — a non-strict truthy test that let unconfirmed (FALSE) rows
through, so pending teams appeared in the combined table. Make act return
explicit TRUE/FALSE (matching the per-round builder) and gate every consumer
(eml/tot/nm/sub) with IF(act=TRUE,...).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plattenplausch-sheet.xlsx
+++ b/plattenplausch-sheet.xlsx
@@ -4098,10 +4098,10 @@
         <f>ARRAYFORMULA(IF($B$2:$B$1001="","",SCAN(0,$B$2:$B$1001,LAMBDA(acc,v,IF(v="",acc,acc+1)))))</f>
       </c>
       <c r="B2">
-        <f>IFERROR(LET(act,MAP(Submissions!$C$2:$C$1001,Submissions!$L$2:$L$1001,Submissions!$N$2:$N$1001,LAMBDA(tn,cf,ss,IF(tn="",FALSE,AND(cf=TRUE,ss&lt;&gt;TRUE)))),eml,IF(act,Submissions!$B$2:$B$1001,""),tot,IF(act,IF(Submissions!$D$2:$D$1001="HIN",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores_Hin!$A$2:$A$25,Scores_Hin!$O$2:$O$25),0))))),IF(Submissions!$D$2:$D$1001="RUECK",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores_Rueck!$A$2:$A$25,Scores_Rueck!$O$2:$O$25),0))))),0)),0),nm,IF(act,Submissions!$C$2:$C$1001,""),sub,IF(act,Submissions!$A$2:$A$1001,""),ue,UNIQUE(FILTER(eml,eml&lt;&gt;"")),uTot,MAP(ue,LAMBDA(e,SUMPRODUCT((eml=e)*IF(ISNUMBER(tot),tot,0)))),uName,MAP(ue,LAMBDA(e,INDEX(FILTER(nm,eml=e),1))),uEarl,MAP(ue,LAMBDA(e,MINIFS(sub,eml,e))),sorted,SORT(HSTACK(uName,uTot,uEarl),2,FALSE,3,TRUE,1,TRUE),INDEX(sorted,0,1)),"")</f>
+        <f>IFERROR(LET(act,MAP(Submissions!$C$2:$C$1001,Submissions!$L$2:$L$1001,Submissions!$N$2:$N$1001,LAMBDA(tn,cf,ss,IF(tn="",FALSE,IF(AND(cf=TRUE,ss&lt;&gt;TRUE),TRUE,FALSE)))),eml,IF(act=TRUE,Submissions!$B$2:$B$1001,""),tot,IF(act=TRUE,IF(Submissions!$D$2:$D$1001="HIN",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores_Hin!$A$2:$A$25,Scores_Hin!$O$2:$O$25),0))))),IF(Submissions!$D$2:$D$1001="RUECK",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores_Rueck!$A$2:$A$25,Scores_Rueck!$O$2:$O$25),0))))),0)),0),nm,IF(act=TRUE,Submissions!$C$2:$C$1001,""),sub,IF(act=TRUE,Submissions!$A$2:$A$1001,""),ue,UNIQUE(FILTER(eml,eml&lt;&gt;"")),uTot,MAP(ue,LAMBDA(e,SUMPRODUCT((eml=e)*IF(ISNUMBER(tot),tot,0)))),uName,MAP(ue,LAMBDA(e,INDEX(FILTER(nm,eml=e),1))),uEarl,MAP(ue,LAMBDA(e,MINIFS(sub,eml,e))),sorted,SORT(HSTACK(uName,uTot,uEarl),2,FALSE,3,TRUE,1,TRUE),INDEX(sorted,0,1)),"")</f>
       </c>
       <c r="C2">
-        <f>IFERROR(LET(act,MAP(Submissions!$C$2:$C$1001,Submissions!$L$2:$L$1001,Submissions!$N$2:$N$1001,LAMBDA(tn,cf,ss,IF(tn="",FALSE,AND(cf=TRUE,ss&lt;&gt;TRUE)))),eml,IF(act,Submissions!$B$2:$B$1001,""),tot,IF(act,IF(Submissions!$D$2:$D$1001="HIN",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores_Hin!$A$2:$A$25,Scores_Hin!$O$2:$O$25),0))))),IF(Submissions!$D$2:$D$1001="RUECK",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores_Rueck!$A$2:$A$25,Scores_Rueck!$O$2:$O$25),0))))),0)),0),nm,IF(act,Submissions!$C$2:$C$1001,""),sub,IF(act,Submissions!$A$2:$A$1001,""),ue,UNIQUE(FILTER(eml,eml&lt;&gt;"")),uTot,MAP(ue,LAMBDA(e,SUMPRODUCT((eml=e)*IF(ISNUMBER(tot),tot,0)))),uName,MAP(ue,LAMBDA(e,INDEX(FILTER(nm,eml=e),1))),uEarl,MAP(ue,LAMBDA(e,MINIFS(sub,eml,e))),sorted,SORT(HSTACK(uName,uTot,uEarl),2,FALSE,3,TRUE,1,TRUE),INDEX(sorted,0,2)),"")</f>
+        <f>IFERROR(LET(act,MAP(Submissions!$C$2:$C$1001,Submissions!$L$2:$L$1001,Submissions!$N$2:$N$1001,LAMBDA(tn,cf,ss,IF(tn="",FALSE,IF(AND(cf=TRUE,ss&lt;&gt;TRUE),TRUE,FALSE)))),eml,IF(act=TRUE,Submissions!$B$2:$B$1001,""),tot,IF(act=TRUE,IF(Submissions!$D$2:$D$1001="HIN",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores_Hin!$A$2:$A$25,Scores_Hin!$O$2:$O$25),0))))),IF(Submissions!$D$2:$D$1001="RUECK",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores_Rueck!$A$2:$A$25,Scores_Rueck!$O$2:$O$25),0))))),0)),0),nm,IF(act=TRUE,Submissions!$C$2:$C$1001,""),sub,IF(act=TRUE,Submissions!$A$2:$A$1001,""),ue,UNIQUE(FILTER(eml,eml&lt;&gt;"")),uTot,MAP(ue,LAMBDA(e,SUMPRODUCT((eml=e)*IF(ISNUMBER(tot),tot,0)))),uName,MAP(ue,LAMBDA(e,INDEX(FILTER(nm,eml=e),1))),uEarl,MAP(ue,LAMBDA(e,MINIFS(sub,eml,e))),sorted,SORT(HSTACK(uName,uTot,uEarl),2,FALSE,3,TRUE,1,TRUE),INDEX(sorted,0,2)),"")</f>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(sheet): Gesamt — gate every row element-wise via MAP (real unconfirmed-leak fix)
Root cause: inside LET, a bare IF(actArray=TRUE, rangeA, rangeB) is NOT
element-wise — Sheets evaluates the condition as a single truthy test and
returns the WHOLE rangeA, so unconfirmed rows' emails entered the aggregate and
pending teams showed in Ranking_Gesamt. (Ranking_Hin was unaffected: it filters
a written cell column with FILTER(...,=TRUE).)

Fix: build eml/tot/nm/sub with MAP over the source columns so each row is gated
by its own confirmed/superseded/teamName. Per-row pick totals via INDEX(picks,i,0)
XLOOKUP'd into the round's Scores sheet. Verified in simulation against the live
2-row data: only the confirmed team appears.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plattenplausch-sheet.xlsx
+++ b/plattenplausch-sheet.xlsx
@@ -4098,10 +4098,10 @@
         <f>ARRAYFORMULA(IF($B$2:$B$1001="","",SCAN(0,$B$2:$B$1001,LAMBDA(acc,v,IF(v="",acc,acc+1)))))</f>
       </c>
       <c r="B2">
-        <f>IFERROR(LET(act,MAP(Submissions!$C$2:$C$1001,Submissions!$L$2:$L$1001,Submissions!$N$2:$N$1001,LAMBDA(tn,cf,ss,IF(tn="",FALSE,IF(AND(cf=TRUE,ss&lt;&gt;TRUE),TRUE,FALSE)))),eml,IF(act=TRUE,Submissions!$B$2:$B$1001,""),tot,IF(act=TRUE,IF(Submissions!$D$2:$D$1001="HIN",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores_Hin!$A$2:$A$25,Scores_Hin!$O$2:$O$25),0))))),IF(Submissions!$D$2:$D$1001="RUECK",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores_Rueck!$A$2:$A$25,Scores_Rueck!$O$2:$O$25),0))))),0)),0),nm,IF(act=TRUE,Submissions!$C$2:$C$1001,""),sub,IF(act=TRUE,Submissions!$A$2:$A$1001,""),ue,UNIQUE(FILTER(eml,eml&lt;&gt;"")),uTot,MAP(ue,LAMBDA(e,SUMPRODUCT((eml=e)*IF(ISNUMBER(tot),tot,0)))),uName,MAP(ue,LAMBDA(e,INDEX(FILTER(nm,eml=e),1))),uEarl,MAP(ue,LAMBDA(e,MINIFS(sub,eml,e))),sorted,SORT(HSTACK(uName,uTot,uEarl),2,FALSE,3,TRUE,1,TRUE),INDEX(sorted,0,1)),"")</f>
+        <f>IFERROR(LET(n,ROWS(Submissions!$C$2:$C$1001),idx,SEQUENCE(n),eml,MAP(Submissions!$C$2:$C$1001,Submissions!$L$2:$L$1001,Submissions!$N$2:$N$1001,Submissions!$B$2:$B$1001,LAMBDA(tn,cf,ss,em,IF(AND(tn&lt;&gt;"",cf=TRUE,ss&lt;&gt;TRUE),em,""))),tot,MAP(Submissions!$C$2:$C$1001,Submissions!$L$2:$L$1001,Submissions!$N$2:$N$1001,Submissions!$D$2:$D$1001,idx,LAMBDA(tn,cf,ss,rd,i,IF(AND(tn&lt;&gt;"",cf=TRUE,ss&lt;&gt;TRUE),IF(rd="HIN",SUMPRODUCT(IFERROR(XLOOKUP(INDEX(Submissions!$E$2:$J$1001,i,0),Scores_Hin!$A$2:$A$25,Scores_Hin!$O$2:$O$25),0)),IF(rd="RUECK",SUMPRODUCT(IFERROR(XLOOKUP(INDEX(Submissions!$E$2:$J$1001,i,0),Scores_Rueck!$A$2:$A$25,Scores_Rueck!$O$2:$O$25),0)),0)),0))),nm,MAP(Submissions!$C$2:$C$1001,Submissions!$L$2:$L$1001,Submissions!$N$2:$N$1001,LAMBDA(tn,cf,ss,IF(AND(tn&lt;&gt;"",cf=TRUE,ss&lt;&gt;TRUE),tn,""))),sub,MAP(Submissions!$C$2:$C$1001,Submissions!$L$2:$L$1001,Submissions!$N$2:$N$1001,Submissions!$A$2:$A$1001,LAMBDA(tn,cf,ss,sb,IF(AND(tn&lt;&gt;"",cf=TRUE,ss&lt;&gt;TRUE),sb,""))),ue,UNIQUE(FILTER(eml,eml&lt;&gt;"")),uTot,MAP(ue,LAMBDA(e,SUMPRODUCT((eml=e)*IF(ISNUMBER(tot),tot,0)))),uName,MAP(ue,LAMBDA(e,INDEX(FILTER(nm,eml=e),1))),uEarl,MAP(ue,LAMBDA(e,MINIFS(sub,eml,e))),sorted,SORT(HSTACK(uName,uTot,uEarl),2,FALSE,3,TRUE,1,TRUE),INDEX(sorted,0,1)),"")</f>
       </c>
       <c r="C2">
-        <f>IFERROR(LET(act,MAP(Submissions!$C$2:$C$1001,Submissions!$L$2:$L$1001,Submissions!$N$2:$N$1001,LAMBDA(tn,cf,ss,IF(tn="",FALSE,IF(AND(cf=TRUE,ss&lt;&gt;TRUE),TRUE,FALSE)))),eml,IF(act=TRUE,Submissions!$B$2:$B$1001,""),tot,IF(act=TRUE,IF(Submissions!$D$2:$D$1001="HIN",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores_Hin!$A$2:$A$25,Scores_Hin!$O$2:$O$25),0))))),IF(Submissions!$D$2:$D$1001="RUECK",BYROW(Submissions!$E$2:$J$1001,LAMBDA(row,IF(INDEX(row,1,1)="",0,SUMPRODUCT(IFERROR(XLOOKUP(row,Scores_Rueck!$A$2:$A$25,Scores_Rueck!$O$2:$O$25),0))))),0)),0),nm,IF(act=TRUE,Submissions!$C$2:$C$1001,""),sub,IF(act=TRUE,Submissions!$A$2:$A$1001,""),ue,UNIQUE(FILTER(eml,eml&lt;&gt;"")),uTot,MAP(ue,LAMBDA(e,SUMPRODUCT((eml=e)*IF(ISNUMBER(tot),tot,0)))),uName,MAP(ue,LAMBDA(e,INDEX(FILTER(nm,eml=e),1))),uEarl,MAP(ue,LAMBDA(e,MINIFS(sub,eml,e))),sorted,SORT(HSTACK(uName,uTot,uEarl),2,FALSE,3,TRUE,1,TRUE),INDEX(sorted,0,2)),"")</f>
+        <f>IFERROR(LET(n,ROWS(Submissions!$C$2:$C$1001),idx,SEQUENCE(n),eml,MAP(Submissions!$C$2:$C$1001,Submissions!$L$2:$L$1001,Submissions!$N$2:$N$1001,Submissions!$B$2:$B$1001,LAMBDA(tn,cf,ss,em,IF(AND(tn&lt;&gt;"",cf=TRUE,ss&lt;&gt;TRUE),em,""))),tot,MAP(Submissions!$C$2:$C$1001,Submissions!$L$2:$L$1001,Submissions!$N$2:$N$1001,Submissions!$D$2:$D$1001,idx,LAMBDA(tn,cf,ss,rd,i,IF(AND(tn&lt;&gt;"",cf=TRUE,ss&lt;&gt;TRUE),IF(rd="HIN",SUMPRODUCT(IFERROR(XLOOKUP(INDEX(Submissions!$E$2:$J$1001,i,0),Scores_Hin!$A$2:$A$25,Scores_Hin!$O$2:$O$25),0)),IF(rd="RUECK",SUMPRODUCT(IFERROR(XLOOKUP(INDEX(Submissions!$E$2:$J$1001,i,0),Scores_Rueck!$A$2:$A$25,Scores_Rueck!$O$2:$O$25),0)),0)),0))),nm,MAP(Submissions!$C$2:$C$1001,Submissions!$L$2:$L$1001,Submissions!$N$2:$N$1001,LAMBDA(tn,cf,ss,IF(AND(tn&lt;&gt;"",cf=TRUE,ss&lt;&gt;TRUE),tn,""))),sub,MAP(Submissions!$C$2:$C$1001,Submissions!$L$2:$L$1001,Submissions!$N$2:$N$1001,Submissions!$A$2:$A$1001,LAMBDA(tn,cf,ss,sb,IF(AND(tn&lt;&gt;"",cf=TRUE,ss&lt;&gt;TRUE),sb,""))),ue,UNIQUE(FILTER(eml,eml&lt;&gt;"")),uTot,MAP(ue,LAMBDA(e,SUMPRODUCT((eml=e)*IF(ISNUMBER(tot),tot,0)))),uName,MAP(ue,LAMBDA(e,INDEX(FILTER(nm,eml=e),1))),uEarl,MAP(ue,LAMBDA(e,MINIFS(sub,eml,e))),sorted,SORT(HSTACK(uName,uTot,uEarl),2,FALSE,3,TRUE,1,TRUE),INDEX(sorted,0,2)),"")</f>
       </c>
     </row>
   </sheetData>

</xml_diff>